<commit_message>
Se incorporan varios formularios
</commit_message>
<xml_diff>
--- a/documentos/Control Turnos 012026 (Monica).xlsx
+++ b/documentos/Control Turnos 012026 (Monica).xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\f_cubillos_2\Desktop\Carlos Castillo Rodriguez\Reportes 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DESARROLLOS\Salud\tmp\HPH\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C84850-A793-4A23-9875-E9A6FD0A5D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A678CB30-0327-4E27-A55B-FA371D8A5CEC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja9" sheetId="9" r:id="rId1"/>
@@ -23,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01.2026'!$A$2:$BO$303</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -33,12 +32,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Carlos Castillo</author>
   </authors>
   <commentList>
-    <comment ref="O2" authorId="0" shapeId="0" xr:uid="{538EF55F-B10E-49E7-AD39-108C8BF266B1}">
+    <comment ref="O2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -62,7 +61,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P2" authorId="0" shapeId="0" xr:uid="{159751D5-CFDF-4A16-9619-915E66C59640}">
+    <comment ref="P2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -86,7 +85,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q2" authorId="0" shapeId="0" xr:uid="{66A10405-A03B-4FFD-9505-C7615EE96636}">
+    <comment ref="Q2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -110,7 +109,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R2" authorId="0" shapeId="0" xr:uid="{B54E0745-0AD5-4233-BD36-159B369A892C}">
+    <comment ref="R2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -124,7 +123,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S2" authorId="0" shapeId="0" xr:uid="{29CFF336-F24C-466D-A390-CC6DF7FF343F}">
+    <comment ref="S2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -148,7 +147,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T2" authorId="0" shapeId="0" xr:uid="{309200B1-11F5-4A7C-8EBA-DED1B1999DBE}">
+    <comment ref="T2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -172,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U2" authorId="0" shapeId="0" xr:uid="{5D36706D-09C2-466B-A7DF-FDFEB9B1DF89}">
+    <comment ref="U2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -187,7 +186,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V2" authorId="0" shapeId="0" xr:uid="{6E8F822C-DAB3-4947-A314-4915B98ADC90}">
+    <comment ref="V2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -201,7 +200,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W2" authorId="0" shapeId="0" xr:uid="{4D7A0956-5A52-4A99-AE30-B4F6345E4F49}">
+    <comment ref="W2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -215,7 +214,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X2" authorId="0" shapeId="0" xr:uid="{AD72BD4E-C5D7-4989-B5C2-E84E845DBB86}">
+    <comment ref="X2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -229,7 +228,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y2" authorId="0" shapeId="0" xr:uid="{68A8FAB0-9CE2-4B43-956C-FF18E9310D35}">
+    <comment ref="Y2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -253,7 +252,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z2" authorId="0" shapeId="0" xr:uid="{D8B0C4BF-E36B-4154-9787-50E972182791}">
+    <comment ref="Z2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -267,7 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA2" authorId="0" shapeId="0" xr:uid="{C4C5F907-20B7-4020-9904-3B21175B680A}">
+    <comment ref="AA2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -291,7 +290,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB2" authorId="0" shapeId="0" xr:uid="{1FA6B3DA-8F5A-4D89-AF73-93ECD9C1B7E9}">
+    <comment ref="AB2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -315,7 +314,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC2" authorId="0" shapeId="0" xr:uid="{5026DD18-C763-4BBA-BB3E-595324F590C5}">
+    <comment ref="AC2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -329,7 +328,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD2" authorId="0" shapeId="0" xr:uid="{F26E7E91-904B-493B-BEB9-488AC7CE73C5}">
+    <comment ref="AD2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -343,7 +342,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE2" authorId="0" shapeId="0" xr:uid="{D556F782-D3D6-4CCF-A26B-3207531180B4}">
+    <comment ref="AE2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -367,7 +366,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF2" authorId="0" shapeId="0" xr:uid="{F4CA8E00-88D7-4FFA-AC33-FDDFDA9A4137}">
+    <comment ref="AF2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -391,7 +390,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG2" authorId="0" shapeId="0" xr:uid="{5E761651-0A6E-47AD-AED5-DAF7BACCB11E}">
+    <comment ref="AG2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -415,7 +414,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH2" authorId="0" shapeId="0" xr:uid="{3141CB71-9E62-4C41-BB72-328323185C85}">
+    <comment ref="AH2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -429,7 +428,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI2" authorId="0" shapeId="0" xr:uid="{14AF2F88-AB3B-4782-B442-6503AC78CD87}">
+    <comment ref="AI2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -453,7 +452,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ2" authorId="0" shapeId="0" xr:uid="{BEAD5DB4-E565-4CB4-BB92-7A2D54C659EE}">
+    <comment ref="AJ2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -467,7 +466,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK2" authorId="0" shapeId="0" xr:uid="{7CE654E5-F055-4555-AA79-8564CD7D180D}">
+    <comment ref="AK2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -481,7 +480,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL2" authorId="0" shapeId="0" xr:uid="{97F3AD00-61A9-483B-8178-370770D385E4}">
+    <comment ref="AL2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -495,7 +494,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AM2" authorId="0" shapeId="0" xr:uid="{6CB99592-E525-46A9-97CB-F1A8A5123DD8}">
+    <comment ref="AM2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -509,7 +508,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN2" authorId="0" shapeId="0" xr:uid="{B525846E-C29D-4610-AB90-C3A11D818655}">
+    <comment ref="AN2" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -523,7 +522,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O309" authorId="0" shapeId="0" xr:uid="{DF05F46C-E6F5-46FF-B503-21C1EAABAFB6}">
+    <comment ref="O309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -547,7 +546,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P309" authorId="0" shapeId="0" xr:uid="{9DE789CF-55BA-4377-A3C1-13FB0AC0028C}">
+    <comment ref="P309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -571,7 +570,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q309" authorId="0" shapeId="0" xr:uid="{48935AE9-E016-49AF-A5D5-1B89E2CDBAE3}">
+    <comment ref="Q309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -595,7 +594,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R309" authorId="0" shapeId="0" xr:uid="{787529E6-E046-4066-9EEA-4F283B3A8164}">
+    <comment ref="R309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -609,7 +608,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S309" authorId="0" shapeId="0" xr:uid="{C3C4DDC9-24D3-4CE1-BB6C-695CB087AD43}">
+    <comment ref="S309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -633,7 +632,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T309" authorId="0" shapeId="0" xr:uid="{AA814B1F-8FFD-4908-8F56-42DFCF70B537}">
+    <comment ref="T309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -657,7 +656,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U309" authorId="0" shapeId="0" xr:uid="{8C2B0258-FF5D-4189-99C6-3C0F3F5D39F6}">
+    <comment ref="U309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -672,7 +671,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V309" authorId="0" shapeId="0" xr:uid="{3C91735F-D59D-46AC-BDE9-5939223E998A}">
+    <comment ref="V309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -686,7 +685,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W309" authorId="0" shapeId="0" xr:uid="{E7B01F25-F85B-4E53-98C9-8B72AC03B61C}">
+    <comment ref="W309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -700,7 +699,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X309" authorId="0" shapeId="0" xr:uid="{8675856F-E894-4051-878F-B35E1FCF4032}">
+    <comment ref="X309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -714,7 +713,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y309" authorId="0" shapeId="0" xr:uid="{0E478627-35A8-4077-8972-8DF14775D202}">
+    <comment ref="Y309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -738,7 +737,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z309" authorId="0" shapeId="0" xr:uid="{B02B6F4F-DE52-4EFA-8BE6-875255F92F24}">
+    <comment ref="Z309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -752,7 +751,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA309" authorId="0" shapeId="0" xr:uid="{0C46CFF2-C95D-494A-BB85-D512E9BCDAF9}">
+    <comment ref="AA309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -776,7 +775,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB309" authorId="0" shapeId="0" xr:uid="{8E48D71C-D5E8-433A-848F-C7396EB9E49C}">
+    <comment ref="AB309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -800,7 +799,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC309" authorId="0" shapeId="0" xr:uid="{0B45452B-F89A-4E2A-9AE4-EB384220E276}">
+    <comment ref="AC309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -814,7 +813,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD309" authorId="0" shapeId="0" xr:uid="{5F8F70F9-2C0C-46E3-AEA0-CE42DD75A630}">
+    <comment ref="AD309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -828,7 +827,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE309" authorId="0" shapeId="0" xr:uid="{A7C376F3-A069-4FD5-B510-FEBDF6E47DE0}">
+    <comment ref="AE309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -852,7 +851,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF309" authorId="0" shapeId="0" xr:uid="{B64DA20A-9215-4069-B26D-41F5B275BA63}">
+    <comment ref="AF309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -876,7 +875,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG309" authorId="0" shapeId="0" xr:uid="{E24B6BFE-E803-40A9-B8A3-407F5390BE8C}">
+    <comment ref="AG309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -900,7 +899,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH309" authorId="0" shapeId="0" xr:uid="{CB5EE7AF-ACDF-4131-BB33-7541170C59F3}">
+    <comment ref="AH309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -914,7 +913,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI309" authorId="0" shapeId="0" xr:uid="{7C43A352-67FE-482A-B158-FA7FC8512729}">
+    <comment ref="AI309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -938,7 +937,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ309" authorId="0" shapeId="0" xr:uid="{97A4E7AD-D7FD-4CCE-A862-D1E1AE82E0F3}">
+    <comment ref="AJ309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -952,7 +951,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AK309" authorId="0" shapeId="0" xr:uid="{A928A835-16D6-4016-9F55-6FB3FA5B0E9D}">
+    <comment ref="AK309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -966,7 +965,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AL309" authorId="0" shapeId="0" xr:uid="{F1F26CF8-5B1C-4DB7-9BC4-2F421E807AF1}">
+    <comment ref="AL309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -980,7 +979,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AM309" authorId="0" shapeId="0" xr:uid="{EBBAB5CA-8296-463E-9850-91B7729B7D39}">
+    <comment ref="AM309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -994,7 +993,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN309" authorId="0" shapeId="0" xr:uid="{BA76A1FA-A475-452B-87F7-A6D48784608A}">
+    <comment ref="AN309" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -1013,7 +1012,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4048" uniqueCount="972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4079" uniqueCount="977">
   <si>
     <t>Dia Dialisis</t>
   </si>
@@ -3929,12 +3928,27 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Codigo</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Periodo</t>
+  </si>
+  <si>
+    <t>IdCargo</t>
+  </si>
+  <si>
+    <t>IdValorHra</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="5">
     <numFmt numFmtId="42" formatCode="_ &quot;$&quot;\ * #,##0_ ;_ &quot;$&quot;\ * \-#,##0_ ;_ &quot;$&quot;\ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;$&quot;\ * #,##0.00_ ;_ &quot;$&quot;\ * \-#,##0.00_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
@@ -4382,9 +4396,9 @@
   <cellStyles count="6">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Moneda [0]" xfId="2" builtinId="7"/>
-    <cellStyle name="Moneda [0] 14" xfId="4" xr:uid="{78E6C9E1-9A96-43F4-9A73-D6383D697340}"/>
-    <cellStyle name="Moneda [0] 2" xfId="3" xr:uid="{306A8694-870C-47CD-8626-A075287F9A1F}"/>
-    <cellStyle name="Moneda [0] 8 2" xfId="5" xr:uid="{C3507E3B-5ECA-444E-96BB-1B9D96415C4E}"/>
+    <cellStyle name="Moneda [0] 14" xfId="4"/>
+    <cellStyle name="Moneda [0] 2" xfId="3"/>
+    <cellStyle name="Moneda [0] 8 2" xfId="5"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -4696,7 +4710,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4125A613-E0CD-4326-B7E1-B6ABC9E55633}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:C24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4951,14 +4965,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9DDF817-544D-4021-85DC-2AE61F8612E8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BQ508"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="2" customWidth="1"/>
     <col min="2" max="2" width="21.42578125" style="2" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" style="2" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" style="3" customWidth="1"/>
     <col min="7" max="9" width="11.42578125" style="3" customWidth="1"/>
@@ -33665,7 +33679,7 @@
         <v>1712000</v>
       </c>
       <c r="BM259" s="44">
-        <f t="shared" ref="BM259:BM322" si="8">+BL259-F259</f>
+        <f t="shared" ref="BM259:BM303" si="8">+BL259-F259</f>
         <v>-181333</v>
       </c>
       <c r="BN259" s="35">
@@ -59275,7 +59289,7 @@
         <v>294640</v>
       </c>
       <c r="BM502" s="40">
-        <f t="shared" ref="BM502:BM533" si="23">+BL502-F502</f>
+        <f t="shared" ref="BM502:BM504" si="23">+BL502-F502</f>
         <v>0</v>
       </c>
       <c r="BN502" s="35">
@@ -59811,7 +59825,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:BO504">
+  <sortState ref="A3:BO504">
     <sortCondition descending="1" ref="N3:N504"/>
   </sortState>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -59824,7 +59838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22EBB9BA-0CC2-42C4-94F5-4A680A8EE147}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="6.7109375" defaultRowHeight="12" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -60541,25 +60555,393 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545EA8AD-8711-4BBF-8F3A-1A62BDA7C561}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>972</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="45" t="s">
+        <v>278</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>403</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>411</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>539</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>547</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>552</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>563</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>569</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>583</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>587</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>611</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>666</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>828</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2071AF9-6F12-4184-BD8C-499799B1FFFE}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>974</v>
+      </c>
+      <c r="B1" t="s">
+        <v>975</v>
+      </c>
+      <c r="C1" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2025</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2025</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2025</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2025</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C149185-B169-4185-A85B-A2FC44B27B97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>